<commit_message>
Extend short extract grid date windows to FY end for mid-year lookups.
Add extendGridDates bootstrap; patch ROYAL/USGI local splits so Oct policies MATCH.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/masters/grid_import_split/ROYAL_grid_26-27.xlsx
+++ b/masters/grid_import_split/ROYAL_grid_26-27.xlsx
@@ -776,10 +776,9 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3W</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>1+1</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>MOTOR</t>
@@ -787,29 +786,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>01-09-2026</t>
+          <t>01-04-2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+          <t>31-03-2027</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
           <t>Auto (3W PCV)</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="n">
         <v>0</v>
       </c>
@@ -831,25 +820,16 @@
           <t>North</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr">
         <is>
           <t>State: Madhya Pradesh (full RTO list not expanded against RTO master)</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr">
         <is>
           <t>Source also shows 'Od Disc' = 55% — an OD discount to customer, not mapped to any PI/PO/retention field here. VERIFY if this needs separate handling.</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="n">
         <v>5</v>
       </c>
@@ -858,32 +838,9 @@
           <t>BAC (Base Agency Commission) - basis not labeled in source as OD/Net, VERIFY</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="inlineStr"/>
+      <c r="AQ2" t="n">
+        <v>5</v>
+      </c>
       <c r="BM2" t="inlineStr">
         <is>
           <t>1 policy: MP-17 Rewa (Commercial/PCV/3W/1+1/Package)</t>

</xml_diff>